<commit_message>
Actualización PAE y Toyota
</commit_message>
<xml_diff>
--- a/downloads/base_completa.xlsx
+++ b/downloads/base_completa.xlsx
@@ -356,7 +356,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB42"/>
+  <dimension ref="A1:AB44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="21" max="21" width="20.7109375" style="2" customWidth="1"/>
@@ -3891,7 +3891,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Pan American Energy (PAE)</t>
+          <t>San Matías Pipeline S.A.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4373,6 +4373,131 @@
       <c r="AB42" t="inlineStr">
         <is>
           <t>https://argentina-lng.ypf.com/assets/pdf/ENG-Argentina-LNG-Adhesion-RIGI.pdf; https://www.lanacion.com.ar/economia/un-proyecto-por-us51000-millones-impulsado-por-ypf-solicito-la-adhesion-al-rigi-nid13082026/; https://www.infobae.com/economia/2026/08/13/con-una-inversion-de-usd-50000-millones-ypf-presenta-al-rigi-el-mayor-proyecto-de-su-historia-para-exportar-gas-de-vaca-muerta/; https://dataenergia.ar/gas/argentina-lgn-solicitaron-la-adhesion-formal-al-rigi-para-una-inversion-historica-de-u-s-51-000-millones-202681319370</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Nueva planta dentro del complejo industrial de Toyota en Zárate para producir un vehículo electrificado —descripto por el ministro de Economía como 100% electrificado—, con aproximadamente 70% de la producción destinada a exportación.</t>
+        </is>
+      </c>
+      <c r="D43">
+        <v>42</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Toyota Argentina S.A. (Argentina)</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Tecnología</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Automotriz</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Zárate</t>
+        </is>
+      </c>
+      <c r="M43">
+        <v>1341</v>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="T43">
+        <v>6200</v>
+      </c>
+      <c r="V43" s="2">
+        <v>46295</v>
+      </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>Luis Caputo / Ministerio de Economía (X, 30/09/2026); Reuters (30/09/2026); La Nación / Toyota Argentina (30/09/2026); ARCA / Decreto 105/2026 (19/02/2026)</t>
+        </is>
+      </c>
+      <c r="AB43" t="inlineStr">
+        <is>
+          <t>https://x.com/LuisCaputoAR/status/2105382049758523681; https://www.reuters.com/world/asia-pacific/toyota-invest-134-billion-argentina-production-plant-2026-09-30/; https://www.lanacion.com.ar/autos/toyota-invertira-us1341-millones-para-fabricar-un-nuevo-vehiculo-en-la-argentina-nid30092026/; https://biblioteca.afip.gob.ar/dcp/DEC_C_000749_2024_08_22</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PAE Cerro Dragón</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Desarrollo de recuperación terciaria de petróleo convencional en Cerro Dragón: 22 plantas de inyección de polímeros, perforación de 100 pozos productores e inyectores, adecuación de pozos, intervención de otros 600 pozos productores e infraestructura complementaria de superficie. Producción incremental estimada: 46 millones de barriles de petróleo y 30 BCF de gas natural.</t>
+        </is>
+      </c>
+      <c r="D44">
+        <v>43</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Pan American Energy (PAE) (Argentina)</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Petróleo y Gas</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Upstream</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Chubut</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Área Cerro Dragón, Cuenca del Golfo San Jorge</t>
+        </is>
+      </c>
+      <c r="M44">
+        <v>1200</v>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="V44" s="2">
+        <v>46296</v>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>Gobierno del Chubut (01/10/2026); La Nación / PAE (01/10/2026); Reuters / Luis Caputo (01/10/2026)</t>
+        </is>
+      </c>
+      <c r="AB44" t="inlineStr">
+        <is>
+          <t>https://noticias.chubut.gob.ar/notas/gobierno/5481/torres-encabezo-en-la-sede-de-la-ocde-el-anuncio-de-una-inversion-de-usd-1200-millones-de-pae-para-cerro-dragon.html; https://www.lanacion.com.ar/economia/pan-american-energy-busca-ingresar-al-rigi-con-una-inversion-de-us1200-millones-para-revitalizar-nid01102026/; https://www.reuters.com/business/energy/pae-invest-12-billion-argentina-oil-field-minister-says-2026-10-01/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización Bajo del Choique–La Invernada
</commit_message>
<xml_diff>
--- a/downloads/base_completa.xlsx
+++ b/downloads/base_completa.xlsx
@@ -2123,7 +2123,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Desarrollo no convencional de petróleo y gas en los bloques Bajo del Choique–La Invernada, en Vaca Muerta. Contempla la perforación de más de 600 pozos, plantas de procesamiento, ductos e infraestructura asociada, con objetivos de hasta 100.000 barriles diarios de petróleo y 12 millones de m³ diarios de gas.</t>
+          <t>Exploración, producción, tratamiento y transporte de hidrocarburos en un área aproximada de 400 km² del centro-norte de Neuquén. El alcance comprende 620 pozos horizontales, cuatro plantas de tratamiento temprano (EPF), un oleoducto de 45 km y un gasoducto de 20 km, con capacidad total de 100.000 barriles diarios de petróleo y 12 millones de Sm³ diarios de gas. La primera etapa prevé 206 pozos y las EPF 1 y 2; la segunda, 414 pozos y las EPF 3 y 4.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D17">
@@ -2136,7 +2141,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Pluspetrol Cuenca Neuquina S.R.L.</t>
+          <t>Gas y Petróleo del Neuquén S.A. - Pluspetrol Cuenca Neuquina S.R.L. – Unión Transitoria Exploración y Producción Bajo del Choique – La Invernada</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>30-71920381-3</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2149,6 +2159,11 @@
           <t>Upstream</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Explotación y producción de nuevos desarrollos de hidrocarburos líquidos y gaseosos costa adentro, con instalaciones complementarias de tratamiento y transporte</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>Neuquén</t>
@@ -2156,37 +2171,62 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Patagonia</t>
+          <t>Centro-norte de Neuquén, aproximadamente 40 km al sur de Rincón de los Sauces; Hub Norte de la Cuenca Neuquina</t>
         </is>
       </c>
       <c r="M17">
-        <v>12400</v>
+        <v>12240</v>
       </c>
       <c r="N17">
-        <v>12400</v>
+        <v>12240</v>
+      </c>
+      <c r="P17">
+        <v>635</v>
+      </c>
+      <c r="Q17">
+        <v>892</v>
       </c>
       <c r="R17">
-        <v>0</v>
+        <v>1527</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="T17">
-        <v>6990</v>
+        <v>2301</v>
+      </c>
+      <c r="U17" s="2">
+        <v>47238</v>
       </c>
       <c r="V17" s="2">
-        <v>45771</v>
+        <v>46135</v>
+      </c>
+      <c r="W17" s="2">
+        <v>46275</v>
+      </c>
+      <c r="X17" s="2">
+        <v>46314</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>Res. 1808/2026</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/detalleAviso/primera/349233/20261019</t>
+        </is>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>Globaris; Gobierno de Neuquén; EconoJournal; Luis Caputo; Clarín; La Nación; Bloomberg</t>
+          <t>Res. 1808/2026; Gobierno de la Provincia del Neuquén; Casa Rosada</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>https://www.neuqueninforma.gob.ar/noticias/2026/04/23/256641-neuquen-suma-un-nuevo-megaproyecto-al-rigi-con-apoyo-de-gyp; https://econojournal.com.ar/oilgas/pluspetrol-solicito-la-adhesion-al-rigi-para-el-bloque-bajo-del-choique-la-invernada-con-una-inversion-de-us12-000-millones/; https://x.com/LuisCaputoAR/status/2047621135127269495; https://www.clarin.com/economia/rigi-vaca-muerta-pluspetrol-presento-inversiones-us-12000-millones-campo-compro-exxon_0_gYALiNgXD0.html; https://www.lanacion.com.ar/economia/pluspetrol-y-gyp-obtuvieron-el-rigi-para-un-proyecto-de-us12400-millones-en-vaca-muerta-nid02102026/; https://www.bloomberglinea.com/latinoamerica/argentina/pluspetrol-recibe-luz-verde-del-rigi-para-invertir-us12400-millones-en-vaca-muerta/</t>
+          <t>https://www.argentina.gob.ar/normativa/nacional/norma-431356; https://www.neuqueninforma.gob.ar/noticias/2026/10/19/265814-vaca-muerta-acelera-su-expansion-aprobaron-el-ingreso-al-rigi-de-un-proyecto-de-12-mil-millones-de-dolares; https://www.casarosada.gob.ar/informacion/conferencias/51404-conferencia-de-prensa-del-vocero-presidencial-adrian-ravier-desde-casa-rosada-19-10-2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
actualización proyecto agua rica
</commit_message>
<xml_diff>
--- a/downloads/base_completa.xlsx
+++ b/downloads/base_completa.xlsx
@@ -1432,12 +1432,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Rincón Mining Pty Ltd.</t>
+          <t>RIGI - RINCON MINING PTY LIMITED</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>30-70708643-9</t>
+          <t>30-71899954-1</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -2018,9 +2018,6 @@
       <c r="M15">
         <v>726</v>
       </c>
-      <c r="R15">
-        <v>0</v>
-      </c>
       <c r="S15" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2087,9 +2084,6 @@
       <c r="M16">
         <v>232</v>
       </c>
-      <c r="R16">
-        <v>0</v>
-      </c>
       <c r="S16" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2384,9 +2378,6 @@
       <c r="M19">
         <v>380</v>
       </c>
-      <c r="R19">
-        <v>0</v>
-      </c>
       <c r="S19" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2453,9 +2444,6 @@
       <c r="M20">
         <v>9500</v>
       </c>
-      <c r="R20">
-        <v>0</v>
-      </c>
       <c r="S20" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2520,10 +2508,7 @@
         </is>
       </c>
       <c r="M21">
-        <v>13800</v>
-      </c>
-      <c r="R21">
-        <v>0</v>
+        <v>9500</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
@@ -2591,9 +2576,6 @@
       <c r="M22">
         <v>200</v>
       </c>
-      <c r="R22">
-        <v>0</v>
-      </c>
       <c r="S22" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2657,9 +2639,6 @@
       <c r="M23">
         <v>206</v>
       </c>
-      <c r="R23">
-        <v>0</v>
-      </c>
       <c r="S23" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -2841,9 +2820,6 @@
       <c r="M25">
         <v>4245</v>
       </c>
-      <c r="R25">
-        <v>0</v>
-      </c>
       <c r="S25" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3136,9 +3112,6 @@
       <c r="M28">
         <v>818</v>
       </c>
-      <c r="R28">
-        <v>0</v>
-      </c>
       <c r="S28" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3426,9 +3399,6 @@
       <c r="M31">
         <v>1000</v>
       </c>
-      <c r="R31">
-        <v>0</v>
-      </c>
       <c r="S31" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -3603,9 +3573,6 @@
       <c r="M33">
         <v>273</v>
       </c>
-      <c r="R33">
-        <v>0</v>
-      </c>
       <c r="S33" t="inlineStr">
         <is>
           <t>Rechazado</t>
@@ -3736,12 +3703,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Minera Agua Rica (MARA)</t>
+          <t>Minera Agua Rica</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
           <t>Desarrollo de una mina de cobre, oro, plata y molibdeno en Catamarca, integrando el yacimiento Agua Rica con la infraestructura existente de Alumbrera, ubicada a unos 35 km. El esquema MARA contempla explotación, procesamiento y uso de instalaciones compartidas para producción destinada principalmente a exportación.</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="D35">
@@ -3757,6 +3729,11 @@
           <t>Minera Agua Rica LLC Sucursal Argentina</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>30-70769036-0</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>Minería</t>
@@ -3767,6 +3744,11 @@
           <t>Cobre</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Minerales de primera y segunda categoría del Código de Minería de la Nación (excluidos potasio y litio)</t>
+        </is>
+      </c>
       <c r="K35" t="inlineStr">
         <is>
           <t>Catamarca</t>
@@ -3778,27 +3760,61 @@
         </is>
       </c>
       <c r="M35">
-        <v>4000</v>
+        <v>6394</v>
+      </c>
+      <c r="N35">
+        <v>6393.631995</v>
+      </c>
+      <c r="O35">
+        <v>3310.574165</v>
+      </c>
+      <c r="P35">
+        <v>111.63955213</v>
+      </c>
+      <c r="Q35">
+        <v>659.8944598</v>
       </c>
       <c r="R35">
-        <v>0</v>
+        <v>771.53401193</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="T35">
+        <v>8200</v>
+      </c>
+      <c r="U35" s="2">
+        <v>47118</v>
       </c>
       <c r="V35" s="2">
         <v>45887</v>
       </c>
+      <c r="W35" s="2">
+        <v>46295</v>
+      </c>
+      <c r="X35" s="2">
+        <v>46322</v>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>Res. 1854/2026</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/detalleAviso/primera/349616/20261027</t>
+        </is>
+      </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>Globaris; Glencore; Luis Caputo; Reuters; Infobae; auditoría 2026-08-08</t>
+          <t>Globaris; Glencore; Luis Caputo; Reuters; Res. 1854/2026; Boletín Oficial; TN</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>https://www.glencore.com/media-and-insights/news/glencore-submits-RIGI-applications-in-respect-of-its-argentine-copper-projects; https://x.com/LuisCaputoAR/status/1957458679835594969; https://www.reuters.com/latam/negocio/7X5ZW2SXG5IYNBUILMTT6GMS6U-2025-08-21/; https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/</t>
+          <t>https://www.glencore.com/media-and-insights/news/glencore-submits-RIGI-applications-in-respect-of-its-argentine-copper-projects; https://x.com/LuisCaputoAR/status/1957458679835594969; https://www.reuters.com/latam/negocio/7X5ZW2SXG5IYNBUILMTT6GMS6U-2025-08-21/; https://www.boletinoficial.gob.ar/detalleAviso/primera/349616/20261027; https://www.cda.org.ar/detalle_normativa.php?id=9497; https://tn.com.ar/economia/2026/10/27/el-gobierno-aprobo-el-ingreso-al-rigi-de-un-proyecto-minero-de-us6393-millones-en-catamarca/?outputType=amp</t>
         </is>
       </c>
     </row>
@@ -4188,9 +4204,6 @@
       <c r="M39">
         <v>1151</v>
       </c>
-      <c r="R39">
-        <v>0</v>
-      </c>
       <c r="S39" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4257,9 +4270,6 @@
       <c r="M40">
         <v>25000</v>
       </c>
-      <c r="R40">
-        <v>0</v>
-      </c>
       <c r="S40" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4326,9 +4336,6 @@
       <c r="M41">
         <v>5800</v>
       </c>
-      <c r="R41">
-        <v>0</v>
-      </c>
       <c r="S41" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4395,9 +4402,6 @@
       <c r="M42">
         <v>51000</v>
       </c>
-      <c r="R42">
-        <v>0</v>
-      </c>
       <c r="S42" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4643,9 +4647,6 @@
       <c r="M45">
         <v>2437</v>
       </c>
-      <c r="R45">
-        <v>0</v>
-      </c>
       <c r="S45" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4706,9 +4707,6 @@
           <t>Tratayén, Neuquén</t>
         </is>
       </c>
-      <c r="R46">
-        <v>0</v>
-      </c>
       <c r="S46" t="inlineStr">
         <is>
           <t>En evaluación</t>
@@ -4768,9 +4766,6 @@
         <is>
           <t>Tratayén–Bahía Blanca / Puerto Galván</t>
         </is>
-      </c>
-      <c r="R47">
-        <v>0</v>
       </c>
       <c r="S47" t="inlineStr">
         <is>

</xml_diff>